<commit_message>
Hogar de Refugio: comparación del metrado de evacuación de arquitectura con el plano de señalización
Lector: posición sin textos y edificación con más holgura donde los contornos se traslapan; reparto de
la señal de riesgo eléctrico tomado del metrado de arquitectura; Excel de comparación y sección en la nota.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_SENALIZACION_Y_SEGURIDAD_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_SENALIZACION_Y_SEGURIDAD_HOGAR_REFUGIO.xlsx
@@ -1715,19 +1715,19 @@
         </is>
       </c>
       <c r="D15" s="14" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" s="14" t="n">
         <v>5</v>
       </c>
       <c r="G15" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="14" t="n">
         <v>5</v>
-      </c>
-      <c r="H15" s="14" t="n">
-        <v>4</v>
       </c>
       <c r="I15" s="14" t="n">
         <v>6</v>
@@ -1738,7 +1738,9 @@
       <c r="K15" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="L15" s="14" t="n"/>
+      <c r="L15" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="M15" s="14" t="n"/>
       <c r="N15" s="14" t="n"/>
       <c r="O15" s="15">
@@ -1806,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" s="14" t="n">
         <v>3</v>
@@ -1815,7 +1817,7 @@
         <v>2</v>
       </c>
       <c r="H17" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I17" s="14" t="n">
         <v>4</v>
@@ -1892,19 +1894,35 @@
           <t>und</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="14" t="n"/>
+      <c r="D19" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L19" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="M19" s="14" t="n"/>
-      <c r="N19" s="14" t="n">
-        <v>39</v>
-      </c>
+      <c r="N19" s="14" t="n"/>
       <c r="O19" s="15">
         <f>SUM(D19:N19)</f>
         <v/>
@@ -1918,7 +1936,7 @@
       </c>
       <c r="R19" s="17" t="inlineStr">
         <is>
-          <t>Imagen pegada en el DXF (sin ubicación): 39 imágenes en el espacio modelo; leyenda: 38</t>
+          <t>Imagen pegada en el DXF (sin ubicación): 39 imágenes en el espacio modelo; reparto por edificación del metrado de evacuación de arquitectura; leyenda: 38</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2266,7 @@
         <v>3</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" s="14" t="n">
         <v>3</v>
@@ -2257,7 +2275,7 @@
         <v>2</v>
       </c>
       <c r="H27" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27" s="14" t="n">
         <v>4</v>
@@ -2307,19 +2325,19 @@
         </is>
       </c>
       <c r="D28" s="14" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" s="14" t="n">
         <v>9</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I28" s="14" t="n">
         <v>12</v>
@@ -2486,14 +2504,14 @@
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>1. Cantidad por edificación: cada símbolo de la planta de la lámina SE-S-02 se asigna a la edificación donde está (contorno del bloque de la planta general, con 0.60 m de margen para las señales de fachada); EXT = exteriores (patios, estacionamientos, puntos ecológicos y circulaciones). No se metran las copias de símbolos que están fuera del terreno.</t>
+          <t>1. Cantidad por edificación: cada símbolo de la planta de la lámina SE-S-02 se asigna a la edificación donde está (contorno del bloque de la planta general, con 0.60 m de margen para las señales de fachada; donde los contornos se traslapan en los aleros, la edificación que lo contiene con más holgura); EXT = exteriores (garita de control, patios, estacionamientos, puntos ecológicos y circulaciones). No se metran las copias de símbolos que están fuera del terreno.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>2. SIN UBICAR: la señal de atención riesgo eléctrico es en el DXF una imagen pegada (OLE) que no exporta su ubicación; se metran las 39 imágenes de igual tamaño del espacio modelo (la leyenda indica 38). Se instalan en los tableros y ambientes eléctricos que indica la lámina, en coordinación con el plano de instalaciones eléctricas.</t>
+          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no exporta su ubicación; se metran las 39 imágenes de igual tamaño del espacio modelo (la leyenda indica 38), con el reparto por edificación del metrado de evacuación de arquitectura, que suma lo mismo. Se instalan en los tableros y ambientes eléctricos que indica la lámina.</t>
         </is>
       </c>
     </row>

</xml_diff>